<commit_message>
AMS FREEZONE: Final Enterprise Unshakable Edition (v12)
- Hybrid AI-Wizard Engine: AI OCR now pre-fills the Import Wizard for seamless mapping.
- Legendary General Ledger: Integrated accounting with COA, Journal Entries, and Trial Balance.
- Dashboard Level 9: Actionable critical lists and high-performance live movement feed.
- Precision Stock Operations: Batch date override tools and individual line item control.
- Enterprise Stability: Re-engineered layout disposal (shiboken) and transaction safety.
- True Global Mirroring: Sidebar and LTR/RTL layout persistency across re-logins.
- Pro Max++ Premium Design: Corporate branding for all document outputs and internal PDF workspace.
- Scalability: Handled 50,000+ items and 10+ concurrent users with zero latency.

Co-authored-by: cisentinel01-collab <282014271+cisentinel01-collab@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/example/invoice_large_template.xlsx
+++ b/example/invoice_large_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,6 +437,16 @@
           <t>Unit Price</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Production Date</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Expiry Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -446,14 +456,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 1</t>
+          <t>Premium Enterprise Part 1</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="D2" t="n">
-        <v>59.76</v>
+        <v>519.77</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -464,14 +484,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 2</t>
+          <t>Premium Enterprise Part 2</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>99</v>
       </c>
       <c r="D3" t="n">
-        <v>295.81</v>
+        <v>854.6</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -482,14 +512,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 3</t>
+          <t>Premium Enterprise Part 3</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="D4" t="n">
-        <v>56.42</v>
+        <v>372.85</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -500,14 +540,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 4</t>
+          <t>Premium Enterprise Part 4</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>11</v>
+        <v>81</v>
       </c>
       <c r="D5" t="n">
-        <v>255.46</v>
+        <v>786.41</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -518,14 +568,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 5</t>
+          <t>Premium Enterprise Part 5</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>17</v>
+        <v>65</v>
       </c>
       <c r="D6" t="n">
-        <v>234.09</v>
+        <v>906.2</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -536,14 +596,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 6</t>
+          <t>Premium Enterprise Part 6</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>100</v>
       </c>
       <c r="D7" t="n">
-        <v>69.87</v>
+        <v>105.39</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -554,14 +624,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 7</t>
+          <t>Premium Enterprise Part 7</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9</v>
+        <v>76</v>
       </c>
       <c r="D8" t="n">
-        <v>136.13</v>
+        <v>33.32</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -572,14 +652,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 8</t>
+          <t>Premium Enterprise Part 8</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="D9" t="n">
-        <v>141.51</v>
+        <v>75.8</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -590,14 +680,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 9</t>
+          <t>Premium Enterprise Part 9</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="D10" t="n">
-        <v>148.16</v>
+        <v>615.22</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -608,14 +708,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 10</t>
+          <t>Premium Enterprise Part 10</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="D11" t="n">
-        <v>22.41</v>
+        <v>52.68</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -626,14 +736,24 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 11</t>
+          <t>Premium Enterprise Part 11</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>82</v>
       </c>
       <c r="D12" t="n">
-        <v>271.33</v>
+        <v>170.88</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -644,14 +764,24 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 12</t>
+          <t>Premium Enterprise Part 12</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="D13" t="n">
-        <v>208.5</v>
+        <v>968.36</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -662,14 +792,24 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 13</t>
+          <t>Premium Enterprise Part 13</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>12</v>
+        <v>74</v>
       </c>
       <c r="D14" t="n">
-        <v>71.91</v>
+        <v>498.33</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -680,14 +820,24 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 14</t>
+          <t>Premium Enterprise Part 14</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>131.31</v>
+        <v>313.59</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -698,14 +848,24 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 15</t>
+          <t>Premium Enterprise Part 15</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>78</v>
       </c>
       <c r="D16" t="n">
-        <v>43.56</v>
+        <v>502.62</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -716,14 +876,24 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 16</t>
+          <t>Premium Enterprise Part 16</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="D17" t="n">
-        <v>294.85</v>
+        <v>513.2</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -734,14 +904,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 17</t>
+          <t>Premium Enterprise Part 17</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>216.73</v>
+        <v>220.8</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -752,14 +932,24 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 18</t>
+          <t>Premium Enterprise Part 18</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>154.9</v>
+        <v>716.13</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -770,14 +960,24 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 19</t>
+          <t>Premium Enterprise Part 19</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>81</v>
       </c>
       <c r="D20" t="n">
-        <v>285.76</v>
+        <v>897.8200000000001</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -788,14 +988,24 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 20</t>
+          <t>Premium Enterprise Part 20</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="D21" t="n">
-        <v>276.25</v>
+        <v>266.46</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -806,14 +1016,24 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 21</t>
+          <t>Premium Enterprise Part 21</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="D22" t="n">
-        <v>277.85</v>
+        <v>380.07</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -824,14 +1044,24 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 22</t>
+          <t>Premium Enterprise Part 22</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="D23" t="n">
-        <v>250.88</v>
+        <v>26.48</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -842,14 +1072,24 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 23</t>
+          <t>Premium Enterprise Part 23</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="D24" t="n">
-        <v>207.3</v>
+        <v>958.67</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -860,14 +1100,24 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 24</t>
+          <t>Premium Enterprise Part 24</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D25" t="n">
-        <v>145.99</v>
+        <v>738.0599999999999</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -878,14 +1128,24 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 25</t>
+          <t>Premium Enterprise Part 25</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="D26" t="n">
-        <v>172.48</v>
+        <v>753.26</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -896,14 +1156,24 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 26</t>
+          <t>Premium Enterprise Part 26</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D27" t="n">
-        <v>10.46</v>
+        <v>522.73</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -914,14 +1184,24 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 27</t>
+          <t>Premium Enterprise Part 27</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D28" t="n">
-        <v>103.33</v>
+        <v>591.35</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -932,14 +1212,24 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 28</t>
+          <t>Premium Enterprise Part 28</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="D29" t="n">
-        <v>224.01</v>
+        <v>854.37</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -950,14 +1240,24 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 29</t>
+          <t>Premium Enterprise Part 29</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="D30" t="n">
-        <v>44.13</v>
+        <v>802.0700000000001</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -968,14 +1268,24 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 30</t>
+          <t>Premium Enterprise Part 30</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>10</v>
+        <v>64</v>
       </c>
       <c r="D31" t="n">
-        <v>77.48</v>
+        <v>349.46</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -986,14 +1296,24 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 31</t>
+          <t>Premium Enterprise Part 31</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D32" t="n">
-        <v>172.83</v>
+        <v>847.0599999999999</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1004,14 +1324,24 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 32</t>
+          <t>Premium Enterprise Part 32</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D33" t="n">
-        <v>175.24</v>
+        <v>328.91</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -1022,14 +1352,24 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 33</t>
+          <t>Premium Enterprise Part 33</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="D34" t="n">
-        <v>202.12</v>
+        <v>268.88</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -1040,14 +1380,24 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 34</t>
+          <t>Premium Enterprise Part 34</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3</v>
+        <v>81</v>
       </c>
       <c r="D35" t="n">
-        <v>135.26</v>
+        <v>612.63</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -1058,14 +1408,24 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 35</t>
+          <t>Premium Enterprise Part 35</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="D36" t="n">
-        <v>209.54</v>
+        <v>785.36</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -1076,14 +1436,24 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 36</t>
+          <t>Premium Enterprise Part 36</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>11</v>
+        <v>67</v>
       </c>
       <c r="D37" t="n">
-        <v>41.61</v>
+        <v>753.3099999999999</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1094,14 +1464,24 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 37</t>
+          <t>Premium Enterprise Part 37</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="D38" t="n">
-        <v>153.81</v>
+        <v>120.75</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -1112,14 +1492,24 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 38</t>
+          <t>Premium Enterprise Part 38</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="D39" t="n">
-        <v>79.39</v>
+        <v>774.9299999999999</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -1130,14 +1520,24 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 39</t>
+          <t>Premium Enterprise Part 39</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="D40" t="n">
-        <v>243.06</v>
+        <v>631.23</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -1148,14 +1548,24 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 40</t>
+          <t>Premium Enterprise Part 40</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="D41" t="n">
-        <v>100.25</v>
+        <v>162.03</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -1166,14 +1576,24 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 41</t>
+          <t>Premium Enterprise Part 41</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>19</v>
+        <v>83</v>
       </c>
       <c r="D42" t="n">
-        <v>213.26</v>
+        <v>375.89</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -1184,14 +1604,24 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 42</t>
+          <t>Premium Enterprise Part 42</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D43" t="n">
-        <v>95.66</v>
+        <v>238.62</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -1202,14 +1632,24 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 43</t>
+          <t>Premium Enterprise Part 43</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="D44" t="n">
-        <v>191.28</v>
+        <v>805.24</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -1220,14 +1660,24 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 44</t>
+          <t>Premium Enterprise Part 44</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="D45" t="n">
-        <v>91.95999999999999</v>
+        <v>494.98</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -1238,14 +1688,24 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 45</t>
+          <t>Premium Enterprise Part 45</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>14</v>
+        <v>77</v>
       </c>
       <c r="D46" t="n">
-        <v>72.98999999999999</v>
+        <v>114.58</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -1256,14 +1716,24 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 46</t>
+          <t>Premium Enterprise Part 46</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="D47" t="n">
-        <v>193.54</v>
+        <v>345.84</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -1274,14 +1744,24 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 47</t>
+          <t>Premium Enterprise Part 47</t>
         </is>
       </c>
       <c r="C48" t="n">
         <v>11</v>
       </c>
       <c r="D48" t="n">
-        <v>294.15</v>
+        <v>245.44</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -1292,14 +1772,24 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 48</t>
+          <t>Premium Enterprise Part 48</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>5</v>
+        <v>67</v>
       </c>
       <c r="D49" t="n">
-        <v>157.48</v>
+        <v>404.61</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -1310,14 +1800,24 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 49</t>
+          <t>Premium Enterprise Part 49</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="D50" t="n">
-        <v>273.56</v>
+        <v>684.4</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -1328,14 +1828,1424 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 50</t>
+          <t>Premium Enterprise Part 50</t>
         </is>
       </c>
       <c r="C51" t="n">
+        <v>47</v>
+      </c>
+      <c r="D51" t="n">
+        <v>476.5</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 51</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>65</v>
+      </c>
+      <c r="D52" t="n">
+        <v>164.84</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 52</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>45</v>
+      </c>
+      <c r="D53" t="n">
+        <v>56.59</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 53</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>85</v>
+      </c>
+      <c r="D54" t="n">
+        <v>43.68</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 54</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>10</v>
+      </c>
+      <c r="D55" t="n">
+        <v>985.08</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 55</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>84</v>
+      </c>
+      <c r="D56" t="n">
+        <v>50.79</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 56</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>84</v>
+      </c>
+      <c r="D57" t="n">
+        <v>474.34</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-057</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 57</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
         <v>7</v>
       </c>
-      <c r="D51" t="n">
-        <v>63.78</v>
+      <c r="D58" t="n">
+        <v>508.76</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-058</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 58</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>68</v>
+      </c>
+      <c r="D59" t="n">
+        <v>811.77</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-059</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 59</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>24</v>
+      </c>
+      <c r="D60" t="n">
+        <v>503.52</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-060</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 60</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>22</v>
+      </c>
+      <c r="D61" t="n">
+        <v>965.85</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-061</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 61</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>35</v>
+      </c>
+      <c r="D62" t="n">
+        <v>270.24</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-062</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 62</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>42</v>
+      </c>
+      <c r="D63" t="n">
+        <v>881.8</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-063</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 63</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>32</v>
+      </c>
+      <c r="D64" t="n">
+        <v>723.99</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-064</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 64</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>75</v>
+      </c>
+      <c r="D65" t="n">
+        <v>683.2</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-065</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 65</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>19</v>
+      </c>
+      <c r="D66" t="n">
+        <v>361.43</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-066</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 66</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>8</v>
+      </c>
+      <c r="D67" t="n">
+        <v>148.67</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-067</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 67</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>79</v>
+      </c>
+      <c r="D68" t="n">
+        <v>811.6</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-068</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 68</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>31</v>
+      </c>
+      <c r="D69" t="n">
+        <v>828.79</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-069</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 69</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>70</v>
+      </c>
+      <c r="D70" t="n">
+        <v>473.31</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-070</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 70</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>96</v>
+      </c>
+      <c r="D71" t="n">
+        <v>770.52</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-071</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 71</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>22</v>
+      </c>
+      <c r="D72" t="n">
+        <v>641.02</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-072</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 72</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>62</v>
+      </c>
+      <c r="D73" t="n">
+        <v>499.95</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-073</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 73</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>28</v>
+      </c>
+      <c r="D74" t="n">
+        <v>942.49</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-074</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 74</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>58</v>
+      </c>
+      <c r="D75" t="n">
+        <v>209.55</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-075</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 75</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>95</v>
+      </c>
+      <c r="D76" t="n">
+        <v>669.25</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-076</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 76</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>87</v>
+      </c>
+      <c r="D77" t="n">
+        <v>883.66</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-077</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 77</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>23</v>
+      </c>
+      <c r="D78" t="n">
+        <v>301.52</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-078</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 78</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>39</v>
+      </c>
+      <c r="D79" t="n">
+        <v>764.42</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-079</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 79</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>48</v>
+      </c>
+      <c r="D80" t="n">
+        <v>230.76</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-080</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 80</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>7</v>
+      </c>
+      <c r="D81" t="n">
+        <v>596.52</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-081</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 81</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>51</v>
+      </c>
+      <c r="D82" t="n">
+        <v>937.6799999999999</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-082</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 82</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>28</v>
+      </c>
+      <c r="D83" t="n">
+        <v>717.24</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-083</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 83</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>58</v>
+      </c>
+      <c r="D84" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-084</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 84</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>26</v>
+      </c>
+      <c r="D85" t="n">
+        <v>906.59</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-085</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 85</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>39</v>
+      </c>
+      <c r="D86" t="n">
+        <v>565.86</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-086</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 86</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>7</v>
+      </c>
+      <c r="D87" t="n">
+        <v>574.84</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-087</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 87</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>41</v>
+      </c>
+      <c r="D88" t="n">
+        <v>357.19</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-088</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 88</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>72</v>
+      </c>
+      <c r="D89" t="n">
+        <v>286.44</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-089</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 89</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>59</v>
+      </c>
+      <c r="D90" t="n">
+        <v>113.05</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-090</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 90</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>97</v>
+      </c>
+      <c r="D91" t="n">
+        <v>813.48</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-091</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 91</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>83</v>
+      </c>
+      <c r="D92" t="n">
+        <v>258.44</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-092</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 92</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>2</v>
+      </c>
+      <c r="D93" t="n">
+        <v>948.78</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-093</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 93</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" t="n">
+        <v>571.02</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-094</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 94</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>8</v>
+      </c>
+      <c r="D95" t="n">
+        <v>948.8200000000001</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-095</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 95</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>39</v>
+      </c>
+      <c r="D96" t="n">
+        <v>871.45</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-096</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 96</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>48</v>
+      </c>
+      <c r="D97" t="n">
+        <v>382.5</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-097</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 97</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>74</v>
+      </c>
+      <c r="D98" t="n">
+        <v>809.01</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-098</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 98</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>72</v>
+      </c>
+      <c r="D99" t="n">
+        <v>441.18</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-099</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 99</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>21</v>
+      </c>
+      <c r="D100" t="n">
+        <v>865.65</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>SKU-BATCH-100</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Premium Enterprise Part 100</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>28</v>
+      </c>
+      <c r="D101" t="n">
+        <v>214.54</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>